<commit_message>
Auto: Week 29/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W29_2026.xlsx
+++ b/Gulf_Dashboard_W29_2026.xlsx
@@ -998,23 +998,69 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>PRJ-015</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>KKE</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>311-314 Refuse Bunker Super structure up to 35.5m elevation 9 May 26 23 Nov 26 Delay Start
+325-326 Tipping hall Foundation up to ground (Include piling work) 1 Feb 26 9 Jul 26 8 Feb 26 On going
+327 Tipping hall Super structure up to 13m elevation 10 Jul 26 19 Oct 26
+330-335 Boiler Island &amp; Auxiliary Equipment Foundation 5 Nov 25 14 Jul 26 8 Jan 26 On going
+346 Steam Turbine Generator &amp; Electrical Construction 18 Feb 26 3 Mar 27 8 Feb 26 On going
+408 Holding Pond and Emergency PondConstruction 23 May 26 20 Nov 26
+14 Boiler Arrival at site 12 Jun 26 12 Jun 26
+11 Incinerator Arrival at site 8 May 26 8 May 26 3 May 26 5 May 26 Completed
+15 Steam turbine Arrival at site 2 Oct 26 2 Oct 26
+62- Producing qualified water (Water Receiving date) 23 Feb 27 8 Mar 27
+Stakeholder Management
+Follow up face recognition system
+Follow up foreigner work permit status
+157 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 11 Nov 2025 10
+16 - 22 July
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>(17th Jul 2026) (24th Jul 2026)
+Activities CC/SC (*)
+Plan % Actual % Diff. % Plan % Actual % Diff. % Acc.Plan %
+Engineering 10% 91.68% 53.06% -38.62% 92.55% 59.06% -33.49% 93.41%
+Procurement 40% 83.43% 77.785 -5.65% 84.78% 79.51% -5.27% 86.23%
+Construction 40% 22.10% 18.25% -3.85% 23.65% 19.59% -4.06% 25.39%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 51.38% 43.72% -7.66% 52.62% 45.55% -7.07% 53.99%
+On Schedule A Bit Delay Big Delay EPC has adjusted the PMS to Rev.H to make the plan consistent with the actual work.
+(0.00% or more) (-0.01% to – 4.99%) (-5.00% or more)
+Safety &amp; Health
+Management Weekly Route Walk - Every Tuesday
+Weekly ESH Meeting - Every Tuesday
+Weekly Project Meeting with - Every Tuesday
+Toolbox Talk - Everyday before working
+Safety training (if any)
+Inspect equipment before working (Daily)
+Random test alcohol
+Environment &amp; CoP
+Road cleaning</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1157,42 +1203,132 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>PRJ-019</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>PKP</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Stakeholder Management
+87 Safety Weekly Audit issue status by weekly
+Total Issues 20
+Since 25 Jan 2026
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+Unsafe Condition The condition was improved
+HUASHI: Lifeline was not properly prior to use.
+Government Agencies
+Total of corrective action request EHS issue 1 issue
+Opened 2 issues
+Closed 1 issues
+Closed Open
+No. Date of Discipline Subject Status
+PKP-001-NCR –C -001 9 Mar 26 Civil Embedded Material for Boiler &amp; FGT Delivered does not meet the greed-upon specification Closed
+PKP-001-RFC – C - 001 15 May 26 Civil Request for Clarification on Pile Rig Collapse during Operation of the Causes and Prevention Method Opened
+PKP–002–NCR– S –001 18 Jun. 26 EHS Failure to Implement COP Guidelines in Maintaining the Cleanliness of IEAT Road Opened</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>TRIR 0 Key Lookahead Milestones:
+Bunker Building: Lift 1 (-4.5 to +1.0 EL),on 30-31 Jul (Completed Lift 1)
+Boiler Island Area: Completed Ground Slab and Embedded Plate at Z3–Z4 for Slag Extractor
+Installation
+STG &amp; ECB: Complete Pouring Concrete Footing (38/38) 100%
+Boiler : Incinerator Grate Installation
+Area of Concern:
+Bunker, Boiler Island, FGT : Level 3 Schedule update from CEEC is still pending
+Issue to request HO support:
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 73.31% 51.44% -21.87% 76.66% 57.25% -19.41% 84.83%
+Procurement 40% 72.46% 70.54% -1.92% 73.82% 72.87% -0.95% 75.19%
+Construction 40% 11.44% 7.88% -3.56% 12.87% 9.45% -3.42% 14.19%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 40.89% 36.51% -4.38% 42.34% 38.65% -3.69% 44.23%
+On Schedule A Bit Delay Big Delay EPC has adjusted the PMS to Rev.c to make the plan consistent with the actual work.
+(0.00%or more) (-0.01% to – 4.99%) (-5.00% or more)
+Safety &amp; Health</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>PRJ-020</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>PSD</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Stakeholder Management
+106 Safety Weekly Audit issue status by weekly
+Total Issues
+Since 2 Jan 2026 10
+9 - 15 July
+Safety Weekly Audit issue Status Chart
+Open Closed
+Before After
+Unsafe Condition
+Not allow to use
+STECON : found poor sling
+Change to new ones.
+for using (no hook)
+Government Agencies
+Problem : Electric Pole obstruct Entrance
+ต ำแหน่งเสำไฟฟ้ำเดมิ
+N.= 1602494.440
+E.= 671208.496
+Entrance ต ำแหน่งเสำไฟฟ้ำใหม่
+▪ ทำ หนังสอื แจง้ ทำง กนอ &gt;&gt; กนอ ทำ หนังสอื แจง้ ทำง PEA &gt;&gt; PEA นครหลวง รบั เรอื งดำ เนินกำรตอ่</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Key Lookahead Milestones:
+Bunker Building: Lift 1 (EL. -4.5 to +1.0) scheduled for 1–2 Aug (Lift 1 completed).
+Boiler Island: Handover of Z5–Z6 by the end of this month, followed by Incinerator Installation.
+FGT : Column concrete pouring and soil backfilling up to the ground beam level.
+STG &amp; ECB: Commencement of slab works for the 22 kV SWGR &amp; MCC cable trench
+at EL +0.25.
+Boiler &amp; Incinerator: Completion of Incinerator Installation.
+AREA OF CONCERN :
+Bunker Building , Boiler , FGT civil work : Level 3 Schedule update from CEEC is still pending
+ISSUE TO REQUEST HO SUPPORT : -
+Jul 2026) Jul 2026)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 88.35% 51.89% -36.46% 90.50% 57.80% -32.70% 92.15%
+Procurement 40% 77.49% 75.54% -1.95% 78.91% 77.90% -1.01% 80.66%
+Construction 40% 18.78% 9.87% -8.91% 20.13% 11.60% -8.53% 21.48%
+Commissioning 10% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00% 0.00%
+Overall 100% 47.34% 39.35% -7.99% 48.67% 41.58% -7.09% 50.07%
+On Schedule A Bit Delay Big Delay EPC has adjusted the PMS to Rev.C to make the plan consistent with the actual work.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">

</xml_diff>